<commit_message>
test: extend the reference fixture to four month sheets
The real workbook has May, June, July and August; the fixture had only May
and August, so no rolling period ever fully covered two months with data and
the analytics screen had nothing to compare. June and July now sit between
them, including the mid-year appearance of the Frequency column that the
reference file shows.

All figures remain invented.
</commit_message>
<xml_diff>
--- a/tests/fixtures/reference/budget-reference-layout.xlsx
+++ b/tests/fixtures/reference/budget-reference-layout.xlsx
@@ -5,15 +5,17 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="May" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="August" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Core expenses" state="visible" r:id="rId6"/>
+    <sheet sheetId="2" name="June" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="July" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="August" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Core expenses" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="38">
   <si>
     <t>Monthly budget</t>
   </si>
@@ -90,22 +92,25 @@
     <t>Left over cash for the month</t>
   </si>
   <si>
+    <t>Phone emi (sibling)</t>
+  </si>
+  <si>
+    <t>Credit card cashback</t>
+  </si>
+  <si>
     <t>Frequency</t>
   </si>
   <si>
     <t>Monthly</t>
   </si>
   <si>
-    <t>Phone emi (sibling)</t>
-  </si>
-  <si>
     <t>Previous month leftover salary</t>
   </si>
   <si>
+    <t xml:space="preserve">Every month, full payment </t>
+  </si>
+  <si>
     <t>Smart watch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Every month, full payment </t>
   </si>
   <si>
     <t>Core expenses</t>
@@ -724,7 +729,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="D4:I31"/>
+  <dimension ref="D4:H30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="4" spans="4:7" x14ac:dyDescent="0.25">
@@ -741,7 +746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
         <v>1</v>
       </c>
@@ -749,33 +754,27 @@
         <v>2</v>
       </c>
       <c r="H5" t="s">
-        <v>25</v>
-      </c>
-      <c r="I5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
         <v>4</v>
       </c>
       <c r="E6">
-        <v>65000</v>
+        <v>61000</v>
       </c>
       <c r="F6" t="s">
         <v>5</v>
       </c>
       <c r="G6">
-        <v>10000</v>
-      </c>
-      <c r="H6" t="s">
-        <v>26</v>
-      </c>
-      <c r="I6" s="1">
+        <v>5000</v>
+      </c>
+      <c r="H6" s="1">
         <v>51105</v>
       </c>
     </row>
-    <row r="7" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
         <v>6</v>
       </c>
@@ -783,24 +782,21 @@
         <v>2250</v>
       </c>
       <c r="F7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G7">
         <v>2900</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="1">
+        <v>46419</v>
+      </c>
+    </row>
+    <row r="8" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
         <v>26</v>
       </c>
-      <c r="I7" s="1">
-        <v>46419</v>
-      </c>
-    </row>
-    <row r="8" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D8" t="s">
-        <v>28</v>
-      </c>
       <c r="E8">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
@@ -808,176 +804,144 @@
       <c r="G8">
         <v>3600</v>
       </c>
-      <c r="H8" t="s">
-        <v>26</v>
-      </c>
-      <c r="I8" s="1">
+      <c r="H8" s="1">
         <v>46388</v>
       </c>
     </row>
-    <row r="9" spans="6:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F9" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="G9">
-        <v>2999</v>
-      </c>
-      <c r="H9" t="s">
-        <v>26</v>
-      </c>
-      <c r="I9" s="1">
-        <v>46478</v>
-      </c>
-    </row>
-    <row r="10" spans="6:8" x14ac:dyDescent="0.25">
+        <v>13000</v>
+      </c>
+    </row>
+    <row r="10" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G10">
-        <v>9000</v>
-      </c>
-      <c r="H10" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" spans="6:8" x14ac:dyDescent="0.25">
+        <v>6100</v>
+      </c>
+    </row>
+    <row r="11" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F11" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G11">
-        <v>2400</v>
-      </c>
-      <c r="H11" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="6:8" x14ac:dyDescent="0.25">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="12" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F12" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G12">
-        <v>379</v>
-      </c>
-      <c r="H12" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="13" spans="6:8" x14ac:dyDescent="0.25">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="13" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F13" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G13">
-        <v>749</v>
-      </c>
-      <c r="H13" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="14" spans="6:8" x14ac:dyDescent="0.25">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="14" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D14" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14">
+        <f>SUM(E6:E13)</f>
+        <v>66250</v>
+      </c>
       <c r="F14" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G14">
-        <v>10000</v>
-      </c>
-      <c r="H14" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D15" t="s">
-        <v>15</v>
-      </c>
-      <c r="E15">
-        <f>SUM(E6:E14)</f>
-        <v>67250</v>
-      </c>
-      <c r="F15" t="s">
-        <v>15</v>
-      </c>
-      <c r="G15">
-        <f>SUM(G6:G14)</f>
-        <v>42027</v>
+        <f>SUM(G6:G13)</f>
+        <v>41728</v>
+      </c>
+    </row>
+    <row r="19" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E19" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="20" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E20" t="s">
-        <v>16</v>
-      </c>
-      <c r="F20" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="F20">
+        <f>E14-G14</f>
+        <v>24522</v>
       </c>
     </row>
     <row r="21" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E21" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F21">
-        <f>E15-G15</f>
-        <v>25223</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="22" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E22" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F22">
-        <v>7000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="23" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E23" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F23">
-        <v>5000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="24" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E24" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F24">
-        <v>3000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="25" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E25" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F25">
-        <v>2000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="26" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E26" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F26">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="27" spans="5:6" x14ac:dyDescent="0.25">
-      <c r="E27" t="s">
-        <v>23</v>
-      </c>
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="27" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F27">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="28" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F28">
-        <f>SUM(F22:F27)</f>
+        <f>SUM(F21:F26)</f>
         <v>19500</v>
       </c>
     </row>
-    <row r="31" spans="5:6" x14ac:dyDescent="0.25">
-      <c r="E31" t="s">
+    <row r="30" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E30" t="s">
         <v>24</v>
       </c>
-      <c r="F31">
-        <f>F21-F28</f>
-        <v>5723</v>
+      <c r="F30">
+        <f>F20-F27</f>
+        <v>5022</v>
       </c>
     </row>
   </sheetData>
@@ -988,20 +952,534 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="D4:I30"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="4" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" t="s">
+        <v>0</v>
+      </c>
+      <c r="F4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
+        <v>2</v>
+      </c>
+      <c r="H5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>63500</v>
+      </c>
+      <c r="F6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G6">
+        <v>5000</v>
+      </c>
+      <c r="H6" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="1">
+        <v>51105</v>
+      </c>
+    </row>
+    <row r="7" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7">
+        <v>2250</v>
+      </c>
+      <c r="F7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7">
+        <v>2900</v>
+      </c>
+      <c r="H7" t="s">
+        <v>28</v>
+      </c>
+      <c r="I7" s="1">
+        <v>46419</v>
+      </c>
+    </row>
+    <row r="8" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G8">
+        <v>3600</v>
+      </c>
+      <c r="H8" t="s">
+        <v>28</v>
+      </c>
+      <c r="I8" s="1">
+        <v>46388</v>
+      </c>
+    </row>
+    <row r="9" spans="6:8" x14ac:dyDescent="0.25">
+      <c r="F9" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9">
+        <v>5650</v>
+      </c>
+      <c r="H9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="6:8" x14ac:dyDescent="0.25">
+      <c r="F10" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10">
+        <v>5651</v>
+      </c>
+      <c r="H10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="6:8" x14ac:dyDescent="0.25">
+      <c r="F11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11">
+        <v>379</v>
+      </c>
+      <c r="H11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="6:8" x14ac:dyDescent="0.25">
+      <c r="F12" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12">
+        <v>749</v>
+      </c>
+      <c r="H12" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="6:8" x14ac:dyDescent="0.25">
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13">
+        <v>10000</v>
+      </c>
+      <c r="H13" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D14" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14">
+        <f>SUM(E6:E13)</f>
+        <v>65750</v>
+      </c>
+      <c r="F14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G14">
+        <f>SUM(G6:G13)</f>
+        <v>33929</v>
+      </c>
+    </row>
+    <row r="19" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E19" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E20" t="s">
+        <v>17</v>
+      </c>
+      <c r="F20">
+        <f>E14-G14</f>
+        <v>31821</v>
+      </c>
+    </row>
+    <row r="21" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E21" t="s">
+        <v>18</v>
+      </c>
+      <c r="F21">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="22" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E22" t="s">
+        <v>19</v>
+      </c>
+      <c r="F22">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="23" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E23" t="s">
+        <v>20</v>
+      </c>
+      <c r="F23">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="24" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E24" t="s">
+        <v>21</v>
+      </c>
+      <c r="F24">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="25" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E25" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="26" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E26" t="s">
+        <v>23</v>
+      </c>
+      <c r="F26">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="27" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F27">
+        <f>SUM(F21:F26)</f>
+        <v>19500</v>
+      </c>
+    </row>
+    <row r="30" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E30" t="s">
+        <v>24</v>
+      </c>
+      <c r="F30">
+        <f>F20-F27</f>
+        <v>12321</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="D4:I31"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="4" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" t="s">
+        <v>0</v>
+      </c>
+      <c r="F4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
+        <v>2</v>
+      </c>
+      <c r="H5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>65000</v>
+      </c>
+      <c r="F6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G6">
+        <v>10000</v>
+      </c>
+      <c r="H6" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="1">
+        <v>51105</v>
+      </c>
+    </row>
+    <row r="7" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7">
+        <v>2250</v>
+      </c>
+      <c r="F7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7">
+        <v>2900</v>
+      </c>
+      <c r="H7" t="s">
+        <v>28</v>
+      </c>
+      <c r="I7" s="1">
+        <v>46419</v>
+      </c>
+    </row>
+    <row r="8" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G8">
+        <v>3600</v>
+      </c>
+      <c r="H8" t="s">
+        <v>28</v>
+      </c>
+      <c r="I8" s="1">
+        <v>46388</v>
+      </c>
+    </row>
+    <row r="9" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F9" t="s">
+        <v>31</v>
+      </c>
+      <c r="G9">
+        <v>2999</v>
+      </c>
+      <c r="H9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I9" s="1">
+        <v>46478</v>
+      </c>
+    </row>
+    <row r="10" spans="6:8" x14ac:dyDescent="0.25">
+      <c r="F10" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10">
+        <v>9000</v>
+      </c>
+      <c r="H10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="6:8" x14ac:dyDescent="0.25">
+      <c r="F11" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11">
+        <v>2400</v>
+      </c>
+      <c r="H11" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="6:8" x14ac:dyDescent="0.25">
+      <c r="F12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12">
+        <v>379</v>
+      </c>
+      <c r="H12" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="6:8" x14ac:dyDescent="0.25">
+      <c r="F13" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13">
+        <v>749</v>
+      </c>
+      <c r="H13" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="6:8" x14ac:dyDescent="0.25">
+      <c r="F14" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14">
+        <v>10000</v>
+      </c>
+      <c r="H14" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D15" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15">
+        <f>SUM(E6:E14)</f>
+        <v>67250</v>
+      </c>
+      <c r="F15" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15">
+        <f>SUM(G6:G14)</f>
+        <v>42027</v>
+      </c>
+    </row>
+    <row r="20" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E20" t="s">
+        <v>16</v>
+      </c>
+      <c r="F20" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E21" t="s">
+        <v>17</v>
+      </c>
+      <c r="F21">
+        <f>E15-G15</f>
+        <v>25223</v>
+      </c>
+    </row>
+    <row r="22" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E22" t="s">
+        <v>18</v>
+      </c>
+      <c r="F22">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="23" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E23" t="s">
+        <v>19</v>
+      </c>
+      <c r="F23">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="24" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E24" t="s">
+        <v>20</v>
+      </c>
+      <c r="F24">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="25" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E25" t="s">
+        <v>21</v>
+      </c>
+      <c r="F25">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="26" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E26" t="s">
+        <v>22</v>
+      </c>
+      <c r="F26">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="27" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E27" t="s">
+        <v>23</v>
+      </c>
+      <c r="F27">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="28" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F28">
+        <f>SUM(F22:F27)</f>
+        <v>19500</v>
+      </c>
+    </row>
+    <row r="31" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E31" t="s">
+        <v>24</v>
+      </c>
+      <c r="F31">
+        <f>F21-F28</f>
+        <v>5723</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B4:G7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="4" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C5">
         <v>5000</v>
@@ -1012,7 +1490,7 @@
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C6">
         <v>3600</v>
@@ -1023,13 +1501,13 @@
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C7">
         <v>2900</v>
       </c>
       <c r="D7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G7" s="1">
         <v>46388</v>

</xml_diff>